<commit_message>
Add ДРР trend sheet (full period vs last week) to ad recommendations
Most campaigns improving: booster-search 16->10% (now profitable),
RL sea toner 26->15% (don't kill), micro-needle VT 168->37%. Lifting
serum stuck at 19%. Refines verdicts: keep booster-search + RL toner,
cut only booster-recommend + VT family.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_ads/ozon_ad_weekly_recommendations_2026-10-05.xlsx
+++ b/outputs/ozon_ads/ozon_ad_weekly_recommendations_2026-10-05.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Все кампании" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ДРР и кластеры" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Рекомендации" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Тренд (полный vs неделя)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -106,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -149,6 +150,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1473,4 +1477,366 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Динамика ДРР: полный период (01.09–05.10) vs последняя неделя (29.09–05.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Почти всё улучшается — реклама оптимизируется. Это меняет решения по пограничным кампаниям.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Товар / кампания</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ДРР полный</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ДРР неделя</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Тренд</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Вывод</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Тонер кремовый</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Поиск</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>↓ лучше</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>🟢 разгонять — ещё лучше</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Пенка Round Lab</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Поиск</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>🟢 разгонять, бюджет мал</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Крем-бустер</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Поиск</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>↓ лучше</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>🟢 вышел в плюс — держать</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Тонер (поиск+рек)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Поиск+рек</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>↑ хуже</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>🟢 держать (чуть хуже, но ок)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Тонер Round Lab морской</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Поиск</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>↓ лучше</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>🟡 резко лучше — НЕ выключать, сток/ставка</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Лифтинг-сыворотка</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Поиск</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>🟡 застряла на 19% — снизить ставку/сток</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Сыворотка микроиглы VT</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Поиск</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>168.2</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>↓ лучше</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>🔴 лучше, но всё ещё минус — выключить</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>VT PDRN Essence</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Поиск</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>↓ лучше</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>🔴 минус — выключить</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Крем-бустер</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Поиск+рек</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>↓ лучше</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>🔴 минус — выключить</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>ГЛАВНОЕ ПО ТРЕНДУ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>1. Крем-бустер в поиске вышел в плюс (16%→10%) — НЕ выключать поиск, только «рекомендации».</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>2. Тонер Round Lab морской резко улучшился (26%→15%) — раньше был кандидат на выключение, теперь почти в плюсе. Не выключать, добить стоком/ставкой.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>3. Лифтинг-сыворотка застряла на ~19% — единственная, что не улучшается. Снизить ставку или проверить сток/карточку.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>4. Выключать только: крем-бустер «рекомендации» (34%), VT PDRN (28%), VT Reedle, сыворотку микроиглы VT (37%) — они и в тренде минус.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>